<commit_message>
[IMP] l10n_it_einvoice_out(_rc): self-invoice TD20
</commit_message>
<xml_diff>
--- a/l10n_it_einvoice_out/tests/data/res_partner.xlsx
+++ b/l10n_it_einvoice_out/tests/data/res_partner.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="245">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.testcompany.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URCROKA</t>
   </si>
   <si>
     <t xml:space="preserve">z0bug.res_partner_1</t>
@@ -1156,8 +1159,12 @@
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
+      <c r="X2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="ALY2" s="1"/>
@@ -1166,24 +1173,24 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>33</v>
@@ -1198,27 +1205,27 @@
         <v>35</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q3" s="3"/>
       <c r="R3" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1226,34 +1233,34 @@
         <v>1</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>35</v>
@@ -1265,22 +1272,22 @@
         <v>35</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1290,27 +1297,27 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>34</v>
@@ -1322,25 +1329,25 @@
         <v>35</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
@@ -1351,29 +1358,29 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>34</v>
@@ -1385,21 +1392,21 @@
         <v>35</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q6" s="3"/>
       <c r="R6" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
@@ -1410,24 +1417,24 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
@@ -1443,46 +1450,48 @@
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="P7" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
+      <c r="X7" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Y7" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Z7" s="3"/>
       <c r="AA7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
@@ -1498,46 +1507,50 @@
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
       <c r="P8" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
-      <c r="Y8" s="3"/>
+      <c r="X8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="Z8" s="3"/>
       <c r="AA8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>33</v>
@@ -1558,17 +1571,17 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U9" s="3"/>
       <c r="V9" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -1577,29 +1590,29 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>35</v>
@@ -1620,7 +1633,7 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1630,27 +1643,27 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>34</v>
@@ -1665,12 +1678,12 @@
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -1683,27 +1696,27 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>35</v>
@@ -1715,22 +1728,22 @@
         <v>35</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="O12" s="3"/>
       <c r="P12" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
@@ -1741,34 +1754,34 @@
         <v>1</v>
       </c>
       <c r="AA12" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>35</v>
@@ -1780,24 +1793,24 @@
         <v>35</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U13" s="3"/>
       <c r="V13" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -1806,34 +1819,34 @@
         <v>1</v>
       </c>
       <c r="AA13" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>35</v>
@@ -1845,10 +1858,10 @@
         <v>35</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1856,11 +1869,11 @@
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U14" s="3"/>
       <c r="V14" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -1869,29 +1882,29 @@
         <v>1</v>
       </c>
       <c r="AA14" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>33</v>
@@ -1906,27 +1919,27 @@
         <v>35</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O15" s="3"/>
       <c r="P15" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q15" s="3"/>
       <c r="R15" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
@@ -1934,31 +1947,31 @@
         <v>1</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Z15" s="3"/>
       <c r="AA15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3" t="s">
@@ -1973,14 +1986,14 @@
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="Q16" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R16" s="3"/>
       <c r="S16" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
@@ -1989,31 +2002,31 @@
         <v>1</v>
       </c>
       <c r="Y16" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Z16" s="3"/>
       <c r="AA16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3" t="s">
@@ -2026,17 +2039,17 @@
         <v>35</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T17" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
@@ -2045,34 +2058,34 @@
         <v>1</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>35</v>
@@ -2084,24 +2097,24 @@
         <v>35</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O18" s="3"/>
       <c r="P18" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q18" s="3"/>
       <c r="R18" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T18" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
@@ -2110,36 +2123,36 @@
         <v>1</v>
       </c>
       <c r="Y18" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>35</v>
@@ -2151,27 +2164,27 @@
         <v>35</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="O19" s="3"/>
       <c r="P19" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q19" s="3"/>
       <c r="R19" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T19" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U19" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
@@ -2179,34 +2192,34 @@
         <v>1</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Z19" s="3"/>
       <c r="AA19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>34</v>
@@ -2218,25 +2231,25 @@
         <v>35</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O20" s="3"/>
       <c r="P20" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T20" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U20" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
@@ -2247,27 +2260,27 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>34</v>
@@ -2279,19 +2292,19 @@
         <v>35</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O21" s="3"/>
       <c r="P21" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
@@ -2304,24 +2317,24 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>33</v>
@@ -2336,26 +2349,26 @@
         <v>35</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O22" s="3"/>
       <c r="P22" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="T22" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U22" s="3"/>
       <c r="V22" s="3"/>
@@ -2364,31 +2377,31 @@
         <v>1</v>
       </c>
       <c r="Y22" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>33</v>
@@ -2403,26 +2416,26 @@
         <v>35</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O23" s="3"/>
       <c r="P23" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="T23" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U23" s="3"/>
       <c r="V23" s="3"/>
@@ -2431,31 +2444,31 @@
         <v>1</v>
       </c>
       <c r="Y23" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z23" s="3"/>
       <c r="AA23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I24" s="3"/>
       <c r="J24" s="3" t="s">
@@ -2468,25 +2481,25 @@
         <v>35</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O24" s="3"/>
       <c r="P24" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
       <c r="S24" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="T24" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U24" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
@@ -2497,27 +2510,27 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>35</v>
@@ -2529,22 +2542,22 @@
         <v>35</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O25" s="3"/>
       <c r="P25" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="Q25" s="3"/>
       <c r="R25" s="3"/>
       <c r="S25" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="T25" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
@@ -2553,34 +2566,34 @@
         <v>1</v>
       </c>
       <c r="Y25" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z25" s="3"/>
       <c r="AA25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>35</v>
@@ -2592,19 +2605,19 @@
         <v>35</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
       <c r="Q26" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="R26" s="3"/>
       <c r="S26" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
@@ -2614,7 +2627,7 @@
         <v>1</v>
       </c>
       <c r="Y26" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Z26" s="3"/>
       <c r="AA26" s="3"/>

</xml_diff>